<commit_message>
02/03/26 bugfixed identified by RS
</commit_message>
<xml_diff>
--- a/assets/program_logic_v6.xlsx
+++ b/assets/program_logic_v6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7100f48b682a1df6/Work/20251027 IEC TC86 Digital Tool/Digital tool/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="305" documentId="13_ncr:1_{FD3D256E-43A5-4E0A-8438-014B95F3FA0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5A7D235-857E-44DF-83DE-1BCFC099A98F}"/>
+  <xr:revisionPtr revIDLastSave="323" documentId="13_ncr:1_{FD3D256E-43A5-4E0A-8438-014B95F3FA0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1815D9FC-8649-4E65-BB83-ED83DD186907}"/>
   <bookViews>
-    <workbookView xWindow="810" yWindow="-120" windowWidth="28110" windowHeight="16440" activeTab="11" xr2:uid="{0D1380F2-B44E-49CB-9379-F623B51E2EAA}"/>
+    <workbookView xWindow="810" yWindow="-120" windowWidth="28110" windowHeight="16440" activeTab="3" xr2:uid="{0D1380F2-B44E-49CB-9379-F623B51E2EAA}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="8" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <sheet name="Filter 2" sheetId="15" r:id="rId10"/>
     <sheet name="Filter 3" sheetId="16" r:id="rId11"/>
     <sheet name="Filter 4" sheetId="19" r:id="rId12"/>
+    <sheet name="Filter 5" sheetId="20" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="123">
   <si>
     <t>Connector type</t>
   </si>
@@ -352,21 +353,6 @@
     <t>IEC 63267-3-1 *d</t>
   </si>
   <si>
-    <t>B (mean ≤ 0,12 dB; at least 97 % ≤ 0,25 dB)</t>
-  </si>
-  <si>
-    <t>C (mean ≤ 0,25 dB; at least 97 % ≤ 0,5 dB)</t>
-  </si>
-  <si>
-    <t>D (mean ≤ 0,5 dB; at least 97% ≤ 1,0 dB)</t>
-  </si>
-  <si>
-    <t>Bm (mean ≤ 0,3 dB; at least 97 % ≤ 0,6 dB)</t>
-  </si>
-  <si>
-    <t>Cm (mean ≤ 0,5 dB; at least 97 % ≤ 1,0 dB)</t>
-  </si>
-  <si>
     <t>Primary coated fibre</t>
   </si>
   <si>
@@ -397,9 +383,6 @@
     <t>Cable type</t>
   </si>
   <si>
-    <t>Mechanical and environmental cable performance (terminated as cable assembly)</t>
-  </si>
-  <si>
     <t>IN1</t>
   </si>
   <si>
@@ -416,6 +399,24 @@
   </si>
   <si>
     <t>IN3</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Bm</t>
+  </si>
+  <si>
+    <t>Cm</t>
+  </si>
+  <si>
+    <t>IN7</t>
+  </si>
+  <si>
+    <t>Mechanical and environmental cable performance</t>
   </si>
 </sst>
 </file>
@@ -1303,7 +1304,7 @@
         <v>54</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1682,13 +1683,13 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B1" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1786,15 +1787,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="B2" t="s">
         <v>45</v>
@@ -1802,7 +1803,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>102</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
         <v>45</v>
@@ -1810,7 +1811,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="B4" t="s">
         <v>45</v>
@@ -1818,7 +1819,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="B5" t="s">
         <v>1</v>
@@ -1826,7 +1827,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
@@ -1848,15 +1849,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="B1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>2</v>
@@ -1864,7 +1865,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>3</v>
@@ -1872,7 +1873,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>4</v>
@@ -1880,7 +1881,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>5</v>
@@ -1888,7 +1889,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>6</v>
@@ -1896,7 +1897,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>7</v>
@@ -1904,7 +1905,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>8</v>
@@ -1912,7 +1913,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>9</v>
@@ -1920,7 +1921,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>10</v>
@@ -1928,7 +1929,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>11</v>
@@ -1936,7 +1937,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>2</v>
@@ -1944,7 +1945,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>3</v>
@@ -1952,7 +1953,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>4</v>
@@ -1960,7 +1961,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>5</v>
@@ -1968,7 +1969,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>6</v>
@@ -1976,7 +1977,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>7</v>
@@ -1984,7 +1985,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>8</v>
@@ -1992,7 +1993,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>9</v>
@@ -2000,7 +2001,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>10</v>
@@ -2008,7 +2009,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>11</v>
@@ -2016,7 +2017,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>2</v>
@@ -2024,7 +2025,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>3</v>
@@ -2032,7 +2033,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>4</v>
@@ -2040,7 +2041,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>5</v>
@@ -2048,7 +2049,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>6</v>
@@ -2056,7 +2057,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>7</v>
@@ -2064,7 +2065,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>8</v>
@@ -2072,7 +2073,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>9</v>
@@ -2080,7 +2081,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>10</v>
@@ -2088,7 +2089,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>11</v>
@@ -2096,7 +2097,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>2</v>
@@ -2104,7 +2105,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>3</v>
@@ -2112,7 +2113,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>4</v>
@@ -2120,7 +2121,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>5</v>
@@ -2128,7 +2129,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>6</v>
@@ -2136,7 +2137,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>7</v>
@@ -2144,7 +2145,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>8</v>
@@ -2152,7 +2153,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>9</v>
@@ -2160,7 +2161,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>10</v>
@@ -2168,10 +2169,55 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{472902C9-8A32-4DC9-BF83-742F54B9DB58}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -2357,7 +2403,7 @@
         <v>45</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2457,22 +2503,22 @@
     <col min="5" max="5" width="59.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D1" s="7"/>
       <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>2</v>
@@ -2483,7 +2529,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>3</v>
@@ -2494,7 +2540,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>4</v>
@@ -2505,7 +2551,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>5</v>
@@ -2516,7 +2562,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>6</v>
@@ -2527,7 +2573,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>7</v>
@@ -2538,7 +2584,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>8</v>
@@ -2549,7 +2595,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>9</v>
@@ -2560,7 +2606,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>10</v>
@@ -2571,7 +2617,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>11</v>
@@ -2582,7 +2628,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>2</v>
@@ -2593,7 +2639,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>3</v>
@@ -2604,7 +2650,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>4</v>
@@ -2615,7 +2661,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>5</v>
@@ -2626,7 +2672,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>6</v>
@@ -2637,7 +2683,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>7</v>
@@ -2648,7 +2694,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>8</v>
@@ -2659,7 +2705,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>9</v>
@@ -2670,7 +2716,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>10</v>
@@ -2681,7 +2727,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>11</v>
@@ -2692,7 +2738,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>2</v>
@@ -2703,7 +2749,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>3</v>
@@ -2714,7 +2760,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>4</v>
@@ -2725,7 +2771,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>5</v>
@@ -2736,7 +2782,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>6</v>
@@ -2747,7 +2793,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>7</v>
@@ -2758,7 +2804,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>8</v>
@@ -2769,7 +2815,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>9</v>
@@ -2780,7 +2826,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>10</v>
@@ -2791,7 +2837,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>11</v>
@@ -2802,7 +2848,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>2</v>
@@ -2813,7 +2859,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>3</v>
@@ -2824,7 +2870,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>4</v>
@@ -2835,51 +2881,51 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>9</v>
@@ -2890,7 +2936,7 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>10</v>
@@ -2901,7 +2947,7 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>11</v>
@@ -3400,10 +3446,10 @@
     </row>
     <row r="2" spans="1:2" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3474,13 +3520,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="C1" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>